<commit_message>
Update lifecycle status: T02, T03 complete
</commit_message>
<xml_diff>
--- a/project-docs/_readable/04b_task_breakdown.xlsx
+++ b/project-docs/_readable/04b_task_breakdown.xlsx
@@ -625,7 +625,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>not_started</t>
+          <t>done</t>
         </is>
       </c>
     </row>
@@ -677,7 +677,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>not_started</t>
+          <t>done</t>
         </is>
       </c>
     </row>

</xml_diff>